<commit_message>
Sync public webpage data
</commit_message>
<xml_diff>
--- a/forecast-results/河北电网披露及电价预估数据-20260916.xlsx
+++ b/forecast-results/河北电网披露及电价预估数据-20260916.xlsx
@@ -7308,7 +7308,7 @@
         <v>3</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>404.3</v>
+        <v>404.4</v>
       </c>
       <c r="E10" s="13" t="n">
         <v>400</v>
@@ -7349,7 +7349,7 @@
         <v>3</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>404.3</v>
+        <v>404.4</v>
       </c>
       <c r="E11" s="13" t="n">
         <v>400</v>
@@ -7390,7 +7390,7 @@
         <v>3</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>404.3</v>
+        <v>404.4</v>
       </c>
       <c r="E12" s="13" t="n">
         <v>400</v>
@@ -7431,7 +7431,7 @@
         <v>3</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>404.3</v>
+        <v>404.4</v>
       </c>
       <c r="E13" s="13" t="n">
         <v>400</v>
@@ -9604,7 +9604,7 @@
         <v>17</v>
       </c>
       <c r="D66" s="13" t="n">
-        <v>398.98</v>
+        <v>398.99</v>
       </c>
       <c r="E66" s="13" t="n">
         <v>380</v>
@@ -9645,7 +9645,7 @@
         <v>17</v>
       </c>
       <c r="D67" s="13" t="n">
-        <v>398.98</v>
+        <v>398.99</v>
       </c>
       <c r="E67" s="13" t="n">
         <v>380</v>
@@ -9686,7 +9686,7 @@
         <v>17</v>
       </c>
       <c r="D68" s="13" t="n">
-        <v>398.98</v>
+        <v>398.99</v>
       </c>
       <c r="E68" s="13" t="n">
         <v>380</v>
@@ -9727,7 +9727,7 @@
         <v>17</v>
       </c>
       <c r="D69" s="13" t="n">
-        <v>398.98</v>
+        <v>398.99</v>
       </c>
       <c r="E69" s="13" t="n">
         <v>380</v>

</xml_diff>